<commit_message>
changed screw terminal signal assignment to be more logical. waived all checked design rule errors. regenerated output files
</commit_message>
<xml_diff>
--- a/Project Outputs for UZ_PER_deskbench_terminal/Rev01/BOM/BOM_JLC-UZ_PER_deskbench_terminal.xlsx
+++ b/Project Outputs for UZ_PER_deskbench_terminal/Rev01/BOM/BOM_JLC-UZ_PER_deskbench_terminal.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GIT\UltraZohm\pcb_design\uz_per_deskbench_terminal\Project Outputs for UZ_PER_deskbench_terminal\Rev01\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{57FA57EA-97F0-4896-9B3D-207FA467648C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{50198486-9158-4B98-9D81-2E3C43AA4930}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="760" yWindow="760" windowWidth="14400" windowHeight="7270" xr2:uid="{5C32A87C-FE99-4F01-9E0E-A0380383884E}"/>
+    <workbookView xWindow="760" yWindow="760" windowWidth="14400" windowHeight="7270" xr2:uid="{BBCF85A5-1A39-4A6C-96A3-12737A7551CF}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM_JLC-UZ_PER_deskbench_termin" sheetId="1" r:id="rId1"/>
@@ -564,7 +564,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49AFE137-AD3F-4F73-BB09-F515372A41EE}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5C64674C-221A-4392-B9CF-5874DFC327C7}">
   <dimension ref="A1:K10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>

</xml_diff>